<commit_message>
Draft team weekly report from verified M1 progress
</commit_message>
<xml_diff>
--- a/docs/metrics/progress.xlsx
+++ b/docs/metrics/progress.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19-25 Oct 2026" sheetId="1" r:id="R95f81ce0626a4acb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19-25 Oct 2026" sheetId="1" r:id="R1fa4dbb4033c4022"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -317,17 +317,17 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="31" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="37" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="37" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="19" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="57" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="58" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>GoodTracker — weekly progress source (19–25 Oct 2026)</x:v>
+        <x:v>GoodTracker — team progress source (19–25 Oct 2026)</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -337,7 +337,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Repository evidence only. Planned outputs are taken from issues and the M1 charter. No hours or completion percentages were recorded.</x:v>
+        <x:v>Weekly issues describe recurring responsibilities. Observed results below are limited to dated repository evidence; missing work is not counted as zero.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -355,127 +355,167 @@
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="9" t="str">
-        <x:v>Work item</x:v>
+        <x:v>Owner / work item</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Planned output / baseline</x:v>
+        <x:v>Planned weekly output</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
         <x:v>Plan source</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Observed result by 25 Oct</x:v>
+        <x:v>Observed result for the week</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
         <x:v>Observed date</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>Evidence / limitation</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="48" customHeight="1">
+        <x:v>Evidence and remaining check</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="52" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>M1 charter</x:v>
+        <x:v>Talha — #22</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>Objectives, scope, constraints and assumptions</x:v>
+        <x:v>Stakeholder decisions and own contribution links</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>Issue #1; M1 due 22 Oct</x:v>
+        <x:v>Weekly issue #22</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>Charter committed</x:v>
+        <x:v>M1 stakeholder analysis committed</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>21 Oct</x:v>
+        <x:v>20 Oct</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
-        <x:v>Commit a3496ca; issue #1. Repository output, not DYS receipt.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="48" customHeight="1">
+        <x:v>9301b96. New feedback or a dated weekly decision not evidenced.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="52" customHeight="1">
       <x:c r="A6" s="12" t="str">
-        <x:v>M1 report</x:v>
+        <x:v>Kerem — #23</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>Official initiation report, Word + PDF</x:v>
+        <x:v>Technical decisions and progress source data</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>Issue #5; M1 due 22 Oct</x:v>
+        <x:v>Weekly issue #23</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>Final report files committed</x:v>
+        <x:v>M1 charter, risk alignment, and report committed</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
         <x:v>21 Oct</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
-        <x:v>Commit f5a161b; issue #5. DYS upload time not verified here.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="48" customHeight="1">
+        <x:v>a3496ca; 6851aab; f5a161b. Decision log and workbook compiled 26 Oct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="52" customHeight="1">
       <x:c r="A7" s="12" t="str">
-        <x:v>Risk alignment</x:v>
+        <x:v>Eylül — #24</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>Initial risk register aligned with product scope</x:v>
+        <x:v>Test and defect evidence; quality review</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
-        <x:v>Issue #4; M1 plan</x:v>
+        <x:v>Weekly issue #24</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>Android/Supabase risk update committed</x:v>
+        <x:v>M1 success criteria committed</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
         <x:v>21 Oct</x:v>
       </x:c>
       <x:c r="F7" s="12" t="str">
-        <x:v>Commit 6851aab; approach-and-risks.md. Risks remain open.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="48" customHeight="1">
+        <x:v>4d9ba27. No executed test or defect result evidenced.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="52" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>Stack validation</x:v>
+        <x:v>Kardelen — #25</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>Small end-to-end prototype before stack commitment</x:v>
+        <x:v>Weekly report coordination and board upkeep</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
+        <x:v>Weekly issue #25</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="str">
+        <x:v>M1 delivery approach and initial risks committed</x:v>
+      </x:c>
+      <x:c r="E8" s="12" t="str">
+        <x:v>21 Oct</x:v>
+      </x:c>
+      <x:c r="F8" s="12" t="str">
+        <x:v>f9e9e7e. Coordination and board updates need confirmation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="52" customHeight="1">
+      <x:c r="A9" s="12" t="str">
+        <x:v>M1 shared output</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="str">
+        <x:v>Charter, success criteria, risks, report files</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="str">
+        <x:v>M1 issues #1–#5; due 22 Oct</x:v>
+      </x:c>
+      <x:c r="D9" s="12" t="str">
+        <x:v>Final Word and PDF files committed</x:v>
+      </x:c>
+      <x:c r="E9" s="12" t="str">
+        <x:v>21 Oct</x:v>
+      </x:c>
+      <x:c r="F9" s="12" t="str">
+        <x:v>f5a161b. Repository output does not establish DYS upload time.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="52" customHeight="1">
+      <x:c r="A10" s="12" t="str">
+        <x:v>Implementation baseline</x:v>
+      </x:c>
+      <x:c r="B10" s="12" t="str">
+        <x:v>Prototype and measured progress after M2 planning</x:v>
+      </x:c>
+      <x:c r="C10" s="12" t="str">
         <x:v>M1 charter; no dated baseline</x:v>
       </x:c>
-      <x:c r="D8" s="12" t="str">
-        <x:v>No working prototype in repository</x:v>
-      </x:c>
-      <x:c r="E8" s="12" t="str">
+      <x:c r="D10" s="12" t="str">
+        <x:v>No working prototype or measured effort in repository</x:v>
+      </x:c>
+      <x:c r="E10" s="12" t="str">
         <x:v>Not recorded</x:v>
       </x:c>
-      <x:c r="F8" s="12" t="str">
-        <x:v>No implementation or test evidence in main through this reporting week.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="1"/>
-      <x:c r="B9" s="1"/>
-      <x:c r="C9" s="1"/>
-      <x:c r="D9" s="1"/>
-      <x:c r="E9" s="1"/>
-      <x:c r="F9" s="1"/>
-    </x:row>
-    <x:row r="10" ht="38" customHeight="1">
-      <x:c r="A10" s="6" t="str">
-        <x:v>Next: agree M2 baseline, owners and estimates; update this sheet with actual dates and evidence as work occurs.</x:v>
-      </x:c>
-      <x:c r="B10" s="6"/>
-      <x:c r="C10" s="6"/>
-      <x:c r="D10" s="6"/>
-      <x:c r="E10" s="6"/>
-      <x:c r="F10" s="6"/>
+      <x:c r="F10" s="12" t="str">
+        <x:v>M2 baseline, estimates, and test evidence still needed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="1"/>
+      <x:c r="B11" s="1"/>
+      <x:c r="C11" s="1"/>
+      <x:c r="D11" s="1"/>
+      <x:c r="E11" s="1"/>
+      <x:c r="F11" s="1"/>
+    </x:row>
+    <x:row r="12" ht="38" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>Team report draft: docs/weekly/2026-W43.md. Confirm unverified Weekly-role activities before DYS submission.</x:v>
+      </x:c>
+      <x:c r="B12" s="6"/>
+      <x:c r="C12" s="6"/>
+      <x:c r="D12" s="6"/>
+      <x:c r="E12" s="6"/>
+      <x:c r="F12" s="6"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
     <x:mergeCell ref="A2:F2"/>
-    <x:mergeCell ref="A10:F10"/>
+    <x:mergeCell ref="A12:F12"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>